<commit_message>
Cotización para Tyler en 7 South Cabin Road con comparación de precios; agregar tu pago y lo que te llevas en los Excel internos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0137o8WSxNvVuvENWjtHj8Xx
</commit_message>
<xml_diff>
--- a/cotizaciones/Cotizacion_juntas_1_Epoxica.xlsx
+++ b/cotizaciones/Cotizacion_juntas_1_Epoxica.xlsx
@@ -615,10 +615,10 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>• 530 ft², 2 personas, 2 días en total (día 1: quitar junta y rejuntar; día 2: lavado a mano y sellado).</t>
+          <t>• 530 ft², 2 personas (tú eres una de ellas), 2 días en total (día 1: quitar junta y rejuntar; día 2: lavado a mano y sellado).</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -813,163 +813,155 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Horas por día</t>
+          <t>De esas personas, cuántas eres tú</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>horas</t>
+          <t>persona</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Estimación: ajusta a tu jornada real.</t>
+          <t>Dato del usuario: tú eres una de las 2 personas que hacen el trabajo.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Pago por hora por persona</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>35</v>
+          <t>Horas por día</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>9</v>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>USD/hora</t>
+          <t>horas</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Estimación: pon lo que pagas a tus trabajadores (o lo que vale tu hora).</t>
+          <t>Estimación: ajusta a tu jornada real.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Contingencia (imprevistos)</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="n">
-        <v>0.1</v>
+          <t>Pago por hora por persona</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>35</v>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>% del costo</t>
+          <t>USD/hora</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Recomendado 10 %: piezas flojas, juntas más profundas, etc.</t>
+          <t>Estimación: pon lo que pagas a tus trabajadores (o lo que vale tu hora).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>Contingencia (imprevistos)</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>% del costo</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Recomendado 10 %: piezas flojas, juntas más profundas, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
           <t>Margen de ganancia deseado</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B13" s="13" t="n">
         <v>0.35</v>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>% del precio</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>20–35 % normal; 35–50 % en trabajos de lujo o remotos.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>MANO DE OBRA (2 días en total, 2 personas)</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Días</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Costo por día</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>Nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Quitar junta vieja y rejuntar</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>días</t>
-        </is>
-      </c>
-      <c r="D16" s="16">
-        <f>$B$8*$B$9*$B$10</f>
-        <v/>
-      </c>
-      <c r="E16" s="16">
-        <f>B16*D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Día 1.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Lavado profundo a mano</t>
+          <t>Quitar junta vieja y rejuntar</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
@@ -977,7 +969,7 @@
         </is>
       </c>
       <c r="D17" s="16">
-        <f>$B$8*$B$9*$B$10</f>
+        <f>$B$8*$B$10*$B$11</f>
         <v/>
       </c>
       <c r="E17" s="16">
@@ -986,14 +978,14 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Día 2 (mañana). Lavado 100 % a mano, sin máquina.</t>
+          <t>Día 1.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Sellado con J26WB (2 manos)</t>
+          <t>Lavado profundo a mano</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
@@ -1005,7 +997,7 @@
         </is>
       </c>
       <c r="D18" s="16">
-        <f>$B$8*$B$9*$B$10</f>
+        <f>$B$8*$B$10*$B$11</f>
         <v/>
       </c>
       <c r="E18" s="16">
@@ -1014,117 +1006,118 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
+          <t>Día 2 (mañana). Lavado 100 % a mano, sin máquina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Sellado con J26WB (2 manos)</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="D19" s="16">
+        <f>$B$8*$B$10*$B$11</f>
+        <v/>
+      </c>
+      <c r="E19" s="16">
+        <f>B19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
           <t>Día 2 (tarde). Revisa en la ficha de la junta cuánto tiempo debe curar antes de sellar.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Subtotal mano de obra</t>
         </is>
       </c>
-      <c r="B19" s="17">
-        <f>SUM(B16:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="B20" s="17">
+        <f>SUM(B17:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>días</t>
         </is>
       </c>
-      <c r="E19" s="18">
-        <f>SUM(E16:E18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="E20" s="18">
+        <f>SUM(E17:E19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>MATERIALES (a precio de tienda)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Precio unitario</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Nota / fuente</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>Junta epóxica (SpectraLOCK Pro / Kerapoxy)</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>unidad (full unit)</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="n">
-        <v>120</v>
-      </c>
-      <c r="E23" s="16">
-        <f>B23*D23</f>
-        <v/>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Estimación: $100–$140 por unidad; 6–12 unidades según tamaño de piedra y junta. Calcula con la calculadora de Laticrete/Mapei.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Pre-sellador / grout release (piedra porosa)</t>
+          <t>Junta epóxica (SpectraLOCK Pro / Kerapoxy)</t>
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>galón</t>
+          <t>unidad (full unit)</t>
         </is>
       </c>
       <c r="D24" s="21" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="E24" s="16">
         <f>B24*D24</f>
@@ -1132,14 +1125,14 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Estimación: $40–$100. Evita que la epóxica manche la piedra.</t>
+          <t>Estimación: $100–$140 por unidad; 6–12 unidades según tamaño de piedra y junta. Calcula con la calculadora de Laticrete/Mapei.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>Limpiador de residuo epóxico, esponjas, llana</t>
+          <t>Pre-sellador / grout release (piedra porosa)</t>
         </is>
       </c>
       <c r="B25" s="20" t="n">
@@ -1147,11 +1140,11 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>galón</t>
         </is>
       </c>
       <c r="D25" s="21" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="E25" s="16">
         <f>B25*D25</f>
@@ -1159,14 +1152,14 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Estimación.</t>
+          <t>Estimación: $40–$100. Evita que la epóxica manche la piedra.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Sellador J26WB</t>
+          <t>Limpiador de residuo epóxico, esponjas, llana</t>
         </is>
       </c>
       <c r="B26" s="20" t="n">
@@ -1174,11 +1167,11 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>cubeta</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="D26" s="21" t="n">
-        <v>400</v>
+        <v>90</v>
       </c>
       <c r="E26" s="16">
         <f>B26*D26</f>
@@ -1186,26 +1179,26 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Precio dado por el usuario: $400 por cubeta. Verifica en la ficha técnica cuántos ft² cubre una cubeta en 2 manos; si no alcanza para 530 ft², sube la cantidad.</t>
+          <t>Estimación.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>Sellador flexible de poliuretano (juntas de expansión)</t>
+          <t>Sellador J26WB</t>
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>cartucho 10 oz</t>
+          <t>cubeta</t>
         </is>
       </c>
       <c r="D27" s="21" t="n">
-        <v>12</v>
+        <v>400</v>
       </c>
       <c r="E27" s="16">
         <f>B27*D27</f>
@@ -1213,26 +1206,26 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Estimación: $8–$15 por cartucho. Para bordes, muros y juntas cada 8–12 ft.</t>
+          <t>Precio dado por el usuario: $400 por cubeta. Verifica en la ficha técnica cuántos ft² cubre una cubeta en 2 manos; si no alcanza para 530 ft², sube la cantidad.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
         <is>
-          <t>Cordón de respaldo (backer rod)</t>
+          <t>Sellador flexible de poliuretano (juntas de expansión)</t>
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>rollo</t>
+          <t>cartucho 10 oz</t>
         </is>
       </c>
       <c r="D28" s="21" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E28" s="16">
         <f>B28*D28</f>
@@ -1240,14 +1233,14 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Estimación: $10–$25.</t>
+          <t>Estimación: $8–$15 por cartucho. Para bordes, muros y juntas cada 8–12 ft.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>Limpiador pH neutro para piedra + cepillos y fibras (lavado a mano)</t>
+          <t>Cordón de respaldo (backer rod)</t>
         </is>
       </c>
       <c r="B29" s="20" t="n">
@@ -1255,11 +1248,11 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>rollo</t>
         </is>
       </c>
       <c r="D29" s="21" t="n">
-        <v>150</v>
+        <v>18</v>
       </c>
       <c r="E29" s="16">
         <f>B29*D29</f>
@@ -1267,14 +1260,14 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Estimación. Lavado 100 % a mano.</t>
+          <t>Estimación: $10–$25.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>Discos/herramienta para quitar junta, cinta, plástico de protección</t>
+          <t>Limpiador pH neutro para piedra + cepillos y fibras (lavado a mano)</t>
         </is>
       </c>
       <c r="B30" s="20" t="n">
@@ -1286,7 +1279,7 @@
         </is>
       </c>
       <c r="D30" s="21" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E30" s="16">
         <f>B30*D30</f>
@@ -1294,108 +1287,108 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
+          <t>Estimación. Lavado 100 % a mano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Discos/herramienta para quitar junta, cinta, plástico de protección</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="E31" s="16">
+        <f>B31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
           <t>Estimación.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Subtotal materiales</t>
         </is>
       </c>
-      <c r="E31" s="18">
-        <f>SUM(E23:E30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="E32" s="18">
+        <f>SUM(E24:E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>OTROS COSTOS</t>
         </is>
       </c>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Precio unitario</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>Gasolina, traslado y comidas</t>
-        </is>
-      </c>
-      <c r="B35" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>viaje</t>
-        </is>
-      </c>
-      <c r="D35" s="21" t="n">
-        <v>400</v>
-      </c>
-      <c r="E35" s="16">
-        <f>B35*D35</f>
-        <v/>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>Estimación para 2 días.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>Hospedaje</t>
+          <t>Gasolina, traslado y comidas</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>noches</t>
+          <t>viaje</t>
         </is>
       </c>
       <c r="D36" s="21" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="E36" s="16">
         <f>B36*D36</f>
@@ -1403,26 +1396,26 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>Estimación. Si vives cerca de Big Sky, pon 0 noches.</t>
+          <t>Estimación para 2 días.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>Seguro / registro de contratista en el club</t>
+          <t>Hospedaje</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>pago</t>
+          <t>noches</t>
         </is>
       </c>
       <c r="D37" s="21" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="E37" s="16">
         <f>B37*D37</f>
@@ -1430,14 +1423,14 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Estimación. El club suele pedir certificado de seguro (COI).</t>
+          <t>Estimación. Si vives cerca de Big Sky, pon 0 noches.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Disposición de residuos</t>
+          <t>Seguro / registro de contratista en el club</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1449,7 +1442,7 @@
         </is>
       </c>
       <c r="D38" s="21" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="E38" s="16">
         <f>B38*D38</f>
@@ -1457,133 +1450,208 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
+          <t>Estimación. El club suele pedir certificado de seguro (COI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Disposición de residuos</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>pago</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E39" s="16">
+        <f>B39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
           <t>Estimación.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Subtotal otros costos</t>
         </is>
       </c>
-      <c r="E39" s="18">
-        <f>SUM(E35:E38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="E40" s="18">
+        <f>SUM(E36:E39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>RESUMEN: COSTO, PRECIO Y GANANCIA</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="14" t="inlineStr">
-        <is>
-          <t>Costo directo (mano de obra + materiales + otros)</t>
-        </is>
-      </c>
-      <c r="E42" s="16">
-        <f>E19+E31+E39</f>
-        <v/>
-      </c>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
+          <t>Costo directo (mano de obra + materiales + otros)</t>
+        </is>
+      </c>
+      <c r="E43" s="16">
+        <f>E20+E32+E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
           <t>Contingencia</t>
         </is>
       </c>
-      <c r="E43" s="16">
-        <f>E42*$B$11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>COSTO TOTAL (lo que te cuesta a ti)</t>
-        </is>
-      </c>
-      <c r="E44" s="23">
-        <f>E42+E43</f>
+      <c r="E44" s="16">
+        <f>E43*$B$12</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="22" t="inlineStr">
         <is>
-          <t>PRECIO DE VENTA (lo que cobras)</t>
+          <t>COSTO TOTAL (lo que te cuesta a ti)</t>
         </is>
       </c>
       <c r="E45" s="23">
-        <f>E44/(1-$B$12)</f>
-        <v/>
-      </c>
-      <c r="F45" s="11" t="inlineStr">
-        <is>
-          <t>Precio = Costo total ÷ (1 − margen). Así el margen sale exacto.</t>
-        </is>
+        <f>E43+E44</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="22" t="inlineStr">
         <is>
+          <t>PRECIO DE VENTA (lo que cobras)</t>
+        </is>
+      </c>
+      <c r="E46" s="23">
+        <f>E45/(1-$B$13)</f>
+        <v/>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>Precio = Costo total ÷ (1 − margen). Así el margen sale exacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
           <t>GANANCIA</t>
         </is>
       </c>
-      <c r="E46" s="23">
-        <f>E45-E44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="14" t="inlineStr">
-        <is>
-          <t>Margen real</t>
-        </is>
-      </c>
-      <c r="E47" s="24">
-        <f>IF(E45=0,0,E46/E45)</f>
-        <v/>
-      </c>
-      <c r="F47" s="11" t="inlineStr">
-        <is>
-          <t>Comprobación: debe ser igual al margen deseado.</t>
-        </is>
+      <c r="E47" s="23">
+        <f>E46-E45</f>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>Precio por ft²</t>
-        </is>
-      </c>
-      <c r="E48" s="16">
-        <f>E45/$B$7</f>
-        <v/>
+          <t>Margen real</t>
+        </is>
+      </c>
+      <c r="E48" s="24">
+        <f>IF(E46=0,0,E47/E46)</f>
+        <v/>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>Comprobación: debe ser igual al margen deseado.</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
         <is>
+          <t>Precio por ft²</t>
+        </is>
+      </c>
+      <c r="E49" s="16">
+        <f>E46/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
           <t>Ganancia por persona por día</t>
         </is>
       </c>
-      <c r="E49" s="16">
-        <f>IF(B19*$B$8=0,0,E46/(B19*$B$8))</f>
-        <v/>
-      </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="E50" s="16">
+        <f>IF(B20*$B$8=0,0,E47/(B20*$B$8))</f>
+        <v/>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
         <is>
           <t>Ganancia ÷ (días × personas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Tu pago como trabajador</t>
+        </is>
+      </c>
+      <c r="E51" s="16">
+        <f>$B$9*$B$10*$B$11*B20</f>
+        <v/>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Lo que te toca de la mano de obra: tus horas × tu pago por hora × días. Ya está incluido en el costo y en el precio al cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t>LO QUE TE LLEVAS TÚ (ganancia + tu pago)</t>
+        </is>
+      </c>
+      <c r="E52" s="23">
+        <f>E47+E51</f>
+        <v/>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>Esto es lo que realmente te queda a ti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>Lo que te llevas si no se usa la contingencia</t>
+        </is>
+      </c>
+      <c r="E53" s="16">
+        <f>E52+E44</f>
+        <v/>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>Si no hay imprevistos, la contingencia también se queda contigo.</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1783,7 @@
         </is>
       </c>
       <c r="B18" s="28">
-        <f>'Costos'!E16*(1+'Costos'!$B$11)/(1-'Costos'!$B$12)</f>
+        <f>'Costos'!E17*(1+'Costos'!$B$12)/(1-'Costos'!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1726,7 +1794,7 @@
         </is>
       </c>
       <c r="B19" s="28">
-        <f>'Costos'!E17*(1+'Costos'!$B$11)/(1-'Costos'!$B$12)</f>
+        <f>'Costos'!E18*(1+'Costos'!$B$12)/(1-'Costos'!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1737,7 +1805,7 @@
         </is>
       </c>
       <c r="B20" s="28">
-        <f>'Costos'!E18*(1+'Costos'!$B$11)/(1-'Costos'!$B$12)</f>
+        <f>'Costos'!E19*(1+'Costos'!$B$12)/(1-'Costos'!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1748,7 +1816,7 @@
         </is>
       </c>
       <c r="B21" s="28">
-        <f>'Costos'!E31*(1+'Costos'!$B$11)/(1-'Costos'!$B$12)</f>
+        <f>'Costos'!E32*(1+'Costos'!$B$12)/(1-'Costos'!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1759,7 +1827,7 @@
         </is>
       </c>
       <c r="B22" s="28">
-        <f>'Costos'!E39*(1+'Costos'!$B$11)/(1-'Costos'!$B$12)</f>
+        <f>'Costos'!E40*(1+'Costos'!$B$12)/(1-'Costos'!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1823,7 +1891,7 @@
         </is>
       </c>
       <c r="B33" s="29">
-        <f>B23-'Costos'!E45</f>
+        <f>B23-'Costos'!E46</f>
         <v/>
       </c>
     </row>

</xml_diff>